<commit_message>
trabajos con el reporte de orden de corte, produccion
</commit_message>
<xml_diff>
--- a/bin/Debug/net9.0-windows/RollosCortados.xlsx
+++ b/bin/Debug/net9.0-windows/RollosCortados.xlsx
@@ -70,160 +70,172 @@
     <x:t>Numero</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">00604                                             </x:t>
-  </x:si>
-  <x:si>
-    <x:t>RI 631/36 PET ARG Chainlink PA WG90</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30211</x:t>
-  </x:si>
-  <x:si>
-    <x:t>42807411</x:t>
+    <x:t xml:space="preserve">06758                                             </x:t>
+  </x:si>
+  <x:si>
+    <x:t>TOP TRANSFER AP904 SK60</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30922</x:t>
+  </x:si>
+  <x:si>
+    <x:t>42805210</x:t>
   </x:si>
   <x:si>
     <x:t>n/t</x:t>
   </x:si>
   <x:si>
-    <x:t>RC30212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30213</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30214</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30215</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30216</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30217</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30218</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30219</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30220</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30221</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30222</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30223</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30224</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30225</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30226</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30227</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30228</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30229</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30230</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30231</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30232</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30233</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30234</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30235</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30236</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30237</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30238</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30239</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30240</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30241</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30242</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30243</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30244</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30245</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30246</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30247</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30248</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30249</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30250</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30251</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30252</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30253</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30254</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30255</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30256</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30257</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30258</x:t>
+    <x:t>RC30923</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30924</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30925</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30926</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30927</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30928</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30929</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30930</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30931</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30932</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30933</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30934</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30935</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30936</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30937</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30938</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30939</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30940</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30941</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30942</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30943</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30944</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30945</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30946</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30947</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30948</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30949</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30950</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30951</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30952</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30953</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30954</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30955</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30956</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30957</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30958</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30959</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30960</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30961</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30962</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30963</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30964</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30965</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30966</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30967</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30968</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30969</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30970</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30971</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30972</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC30973</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -589,12 +601,12 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:R49"/>
+  <x:dimension ref="A1:R53"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="26.424911" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.853482" style="0" customWidth="1"/>
@@ -682,13 +694,13 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F2" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>0</x:v>
@@ -723,13 +735,13 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F3" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>0</x:v>
@@ -764,13 +776,13 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F4" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H4" s="0">
         <x:v>0</x:v>
@@ -805,13 +817,13 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H5" s="0">
         <x:v>0</x:v>
@@ -846,13 +858,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H6" s="0">
         <x:v>0</x:v>
@@ -887,13 +899,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F7" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H7" s="0">
         <x:v>0</x:v>
@@ -928,13 +940,13 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F8" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H8" s="0">
         <x:v>0</x:v>
@@ -969,13 +981,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F9" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H9" s="0">
         <x:v>0</x:v>
@@ -1010,13 +1022,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F10" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H10" s="0">
         <x:v>0</x:v>
@@ -1051,13 +1063,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F11" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H11" s="0">
         <x:v>0</x:v>
@@ -1092,13 +1104,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F12" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H12" s="0">
         <x:v>0</x:v>
@@ -1133,13 +1145,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F13" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H13" s="0">
         <x:v>0</x:v>
@@ -1174,13 +1186,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F14" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H14" s="0">
         <x:v>0</x:v>
@@ -1215,13 +1227,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F15" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H15" s="0">
         <x:v>0</x:v>
@@ -1256,13 +1268,13 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F16" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H16" s="0">
         <x:v>0</x:v>
@@ -1297,13 +1309,13 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F17" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H17" s="0">
         <x:v>0</x:v>
@@ -1338,13 +1350,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F18" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H18" s="0">
         <x:v>0</x:v>
@@ -1379,13 +1391,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F19" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H19" s="0">
         <x:v>0</x:v>
@@ -1420,13 +1432,13 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F20" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H20" s="0">
         <x:v>0</x:v>
@@ -1461,13 +1473,13 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F21" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H21" s="0">
         <x:v>0</x:v>
@@ -1502,13 +1514,13 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F22" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H22" s="0">
         <x:v>0</x:v>
@@ -1543,13 +1555,13 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F23" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H23" s="0">
         <x:v>0</x:v>
@@ -1584,13 +1596,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H24" s="0">
         <x:v>0</x:v>
@@ -1625,13 +1637,13 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F25" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H25" s="0">
         <x:v>0</x:v>
@@ -1666,13 +1678,13 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F26" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H26" s="0">
         <x:v>0</x:v>
@@ -1707,13 +1719,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F27" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H27" s="0">
         <x:v>0</x:v>
@@ -1748,13 +1760,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F28" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H28" s="0">
         <x:v>0</x:v>
@@ -1789,13 +1801,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F29" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H29" s="0">
         <x:v>0</x:v>
@@ -1830,13 +1842,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F30" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H30" s="0">
         <x:v>0</x:v>
@@ -1871,13 +1883,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F31" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H31" s="0">
         <x:v>0</x:v>
@@ -1912,13 +1924,13 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="E32" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F32" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G32" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H32" s="0">
         <x:v>0</x:v>
@@ -1953,13 +1965,13 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="E33" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F33" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G33" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H33" s="0">
         <x:v>0</x:v>
@@ -1994,13 +2006,13 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="E34" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F34" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G34" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H34" s="0">
         <x:v>0</x:v>
@@ -2035,13 +2047,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="E35" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F35" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G35" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H35" s="0">
         <x:v>0</x:v>
@@ -2076,13 +2088,13 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="E36" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F36" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G36" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H36" s="0">
         <x:v>0</x:v>
@@ -2117,13 +2129,13 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="E37" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F37" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G37" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H37" s="0">
         <x:v>0</x:v>
@@ -2158,13 +2170,13 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E38" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F38" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G38" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H38" s="0">
         <x:v>0</x:v>
@@ -2199,13 +2211,13 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="E39" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F39" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G39" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H39" s="0">
         <x:v>0</x:v>
@@ -2240,13 +2252,13 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="E40" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F40" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G40" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H40" s="0">
         <x:v>0</x:v>
@@ -2281,13 +2293,13 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="E41" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F41" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G41" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H41" s="0">
         <x:v>0</x:v>
@@ -2322,13 +2334,13 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="E42" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F42" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G42" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H42" s="0">
         <x:v>0</x:v>
@@ -2363,13 +2375,13 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="E43" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F43" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G43" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H43" s="0">
         <x:v>0</x:v>
@@ -2404,13 +2416,13 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="E44" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F44" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G44" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H44" s="0">
         <x:v>0</x:v>
@@ -2445,13 +2457,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="E45" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F45" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G45" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H45" s="0">
         <x:v>0</x:v>
@@ -2486,13 +2498,13 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="E46" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F46" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G46" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H46" s="0">
         <x:v>0</x:v>
@@ -2527,13 +2539,13 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="E47" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F47" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G47" s="0">
-        <x:v>64.8</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H47" s="0">
         <x:v>0</x:v>
@@ -2568,13 +2580,13 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="E48" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F48" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G48" s="0">
-        <x:v>108</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="H48" s="0">
         <x:v>0</x:v>
@@ -2609,13 +2621,13 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="E49" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F49" s="0">
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G49" s="0">
-        <x:v>43.2</x:v>
+        <x:v>86.4</x:v>
       </x:c>
       <x:c r="H49" s="0">
         <x:v>0</x:v>
@@ -2633,6 +2645,170 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q49" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" spans="1:18">
+      <x:c r="A50" s="0">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B50" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C50" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D50" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="E50" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F50" s="0">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="G50" s="0">
+        <x:v>86.4</x:v>
+      </x:c>
+      <x:c r="H50" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I50" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J50" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M50" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N50" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q50" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" spans="1:18">
+      <x:c r="A51" s="0">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B51" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C51" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D51" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="E51" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F51" s="0">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="G51" s="0">
+        <x:v>86.4</x:v>
+      </x:c>
+      <x:c r="H51" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I51" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J51" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M51" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N51" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q51" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" spans="1:18">
+      <x:c r="A52" s="0">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B52" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C52" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D52" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E52" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F52" s="0">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="G52" s="0">
+        <x:v>64.8</x:v>
+      </x:c>
+      <x:c r="H52" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I52" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J52" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M52" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N52" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q52" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" spans="1:18">
+      <x:c r="A53" s="0">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B53" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C53" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D53" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="E53" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F53" s="0">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="G53" s="0">
+        <x:v>86.4</x:v>
+      </x:c>
+      <x:c r="H53" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I53" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J53" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M53" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N53" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q53" s="0" t="b">
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
trabajos con la orden de corte, relacion,bindingsource,estados del documento
</commit_message>
<xml_diff>
--- a/bin/Debug/net9.0-windows/RollosCortados.xlsx
+++ b/bin/Debug/net9.0-windows/RollosCortados.xlsx
@@ -70,172 +70,19 @@
     <x:t>Numero</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">06758                                             </x:t>
+    <x:t xml:space="preserve">6758                                              </x:t>
   </x:si>
   <x:si>
-    <x:t>TOP TRANSFER AP904 SK60</x:t>
+    <x:t>Top Transfer Premium FSC AP904 WG55</x:t>
   </x:si>
   <x:si>
-    <x:t>RC30922</x:t>
+    <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t>42805210</x:t>
+    <x:t>225100024</x:t>
   </x:si>
   <x:si>
-    <x:t>n/t</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30923</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30924</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30925</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30926</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30927</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30928</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30929</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30930</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30931</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30932</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30933</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30934</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30935</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30936</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30937</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30938</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30939</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30940</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30941</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30942</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30943</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30944</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30945</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30946</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30947</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30948</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30949</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30950</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30951</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30952</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30953</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30954</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30955</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30956</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30957</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30958</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30959</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30960</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30961</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30962</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30963</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30964</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30965</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30966</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30967</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30968</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30969</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30970</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30971</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30972</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC30973</x:t>
+    <x:t>XT901WZ1140</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -601,19 +448,19 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:R53"/>
+  <x:dimension ref="A1:R51"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="26.424911" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25.139196" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.853482" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="4.567768" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="6.567768" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="5.853482" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="9.282054" style="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12.996339" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10.282054" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13.567768" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="6.424911" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="9.567768" style="0" customWidth="1"/>
     <x:col min="13" max="13" width="18.853482" style="0" customWidth="1"/>
@@ -694,13 +541,13 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>0</x:v>
@@ -732,16 +579,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>0</x:v>
@@ -773,16 +620,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H4" s="0">
         <x:v>0</x:v>
@@ -814,16 +661,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H5" s="0">
         <x:v>0</x:v>
@@ -855,16 +702,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H6" s="0">
         <x:v>0</x:v>
@@ -896,16 +743,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H7" s="0">
         <x:v>0</x:v>
@@ -937,16 +784,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H8" s="0">
         <x:v>0</x:v>
@@ -978,16 +825,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H9" s="0">
         <x:v>0</x:v>
@@ -1019,16 +866,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H10" s="0">
         <x:v>0</x:v>
@@ -1060,16 +907,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H11" s="0">
         <x:v>0</x:v>
@@ -1101,16 +948,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H12" s="0">
         <x:v>0</x:v>
@@ -1142,16 +989,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H13" s="0">
         <x:v>0</x:v>
@@ -1183,16 +1030,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H14" s="0">
         <x:v>0</x:v>
@@ -1224,16 +1071,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H15" s="0">
         <x:v>0</x:v>
@@ -1265,16 +1112,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>3</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>64.8</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H16" s="0">
         <x:v>0</x:v>
@@ -1306,16 +1153,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H17" s="0">
         <x:v>0</x:v>
@@ -1347,16 +1194,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H18" s="0">
         <x:v>0</x:v>
@@ -1388,16 +1235,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H19" s="0">
         <x:v>0</x:v>
@@ -1429,16 +1276,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H20" s="0">
         <x:v>0</x:v>
@@ -1470,16 +1317,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H21" s="0">
         <x:v>0</x:v>
@@ -1511,16 +1358,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H22" s="0">
         <x:v>0</x:v>
@@ -1552,16 +1399,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H23" s="0">
         <x:v>0</x:v>
@@ -1593,16 +1440,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H24" s="0">
         <x:v>0</x:v>
@@ -1634,16 +1481,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H25" s="0">
         <x:v>0</x:v>
@@ -1675,16 +1522,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H26" s="0">
         <x:v>0</x:v>
@@ -1716,16 +1563,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H27" s="0">
         <x:v>0</x:v>
@@ -1757,16 +1604,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H28" s="0">
         <x:v>0</x:v>
@@ -1798,16 +1645,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H29" s="0">
         <x:v>0</x:v>
@@ -1839,16 +1686,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H30" s="0">
         <x:v>0</x:v>
@@ -1880,16 +1727,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H31" s="0">
         <x:v>0</x:v>
@@ -1921,16 +1768,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E32" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F32" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G32" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H32" s="0">
         <x:v>0</x:v>
@@ -1962,16 +1809,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E33" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F33" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G33" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H33" s="0">
         <x:v>0</x:v>
@@ -2003,16 +1850,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E34" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F34" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G34" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H34" s="0">
         <x:v>0</x:v>
@@ -2044,16 +1891,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E35" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F35" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G35" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H35" s="0">
         <x:v>0</x:v>
@@ -2085,16 +1932,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E36" s="0">
-        <x:v>3</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F36" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G36" s="0">
-        <x:v>64.8</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H36" s="0">
         <x:v>0</x:v>
@@ -2126,16 +1973,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E37" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F37" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G37" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H37" s="0">
         <x:v>0</x:v>
@@ -2167,16 +2014,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E38" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F38" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G38" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H38" s="0">
         <x:v>0</x:v>
@@ -2208,16 +2055,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E39" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F39" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G39" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H39" s="0">
         <x:v>0</x:v>
@@ -2249,16 +2096,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E40" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F40" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G40" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H40" s="0">
         <x:v>0</x:v>
@@ -2290,16 +2137,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E41" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F41" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G41" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H41" s="0">
         <x:v>0</x:v>
@@ -2331,16 +2178,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E42" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F42" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G42" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H42" s="0">
         <x:v>0</x:v>
@@ -2372,16 +2219,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E43" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F43" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G43" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H43" s="0">
         <x:v>0</x:v>
@@ -2413,16 +2260,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E44" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F44" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G44" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H44" s="0">
         <x:v>0</x:v>
@@ -2454,16 +2301,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E45" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F45" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G45" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H45" s="0">
         <x:v>0</x:v>
@@ -2495,16 +2342,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E46" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F46" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G46" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H46" s="0">
         <x:v>0</x:v>
@@ -2536,16 +2383,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E47" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F47" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G47" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H47" s="0">
         <x:v>0</x:v>
@@ -2577,16 +2424,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E48" s="0">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F48" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G48" s="0">
-        <x:v>64.8</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H48" s="0">
         <x:v>0</x:v>
@@ -2618,16 +2465,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E49" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F49" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G49" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H49" s="0">
         <x:v>0</x:v>
@@ -2659,16 +2506,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D50" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E50" s="0">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F50" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G50" s="0">
-        <x:v>86.4</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="H50" s="0">
         <x:v>0</x:v>
@@ -2700,16 +2547,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D51" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E51" s="0">
-        <x:v>4</x:v>
+        <x:v>19.4</x:v>
       </x:c>
       <x:c r="F51" s="0">
-        <x:v>1800</x:v>
+        <x:v>2100</x:v>
       </x:c>
       <x:c r="G51" s="0">
-        <x:v>86.4</x:v>
+        <x:v>488.88</x:v>
       </x:c>
       <x:c r="H51" s="0">
         <x:v>0</x:v>
@@ -2727,88 +2574,6 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q51" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" spans="1:18">
-      <x:c r="A52" s="0">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="B52" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C52" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D52" s="0" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="E52" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F52" s="0">
-        <x:v>1800</x:v>
-      </x:c>
-      <x:c r="G52" s="0">
-        <x:v>64.8</x:v>
-      </x:c>
-      <x:c r="H52" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I52" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="J52" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="M52" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N52" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q52" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" spans="1:18">
-      <x:c r="A53" s="0">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="B53" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C53" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D53" s="0" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="E53" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F53" s="0">
-        <x:v>1800</x:v>
-      </x:c>
-      <x:c r="G53" s="0">
-        <x:v>86.4</x:v>
-      </x:c>
-      <x:c r="H53" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I53" s="0" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="J53" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="M53" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N53" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q53" s="0" t="b">
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
trabajos con el inventario de master iniciales en la orden de corte
</commit_message>
<xml_diff>
--- a/bin/Debug/net9.0-windows/RollosCortados.xlsx
+++ b/bin/Debug/net9.0-windows/RollosCortados.xlsx
@@ -76,13 +76,160 @@
     <x:t>Top Transfer Premium FSC AP904 WG55</x:t>
   </x:si>
   <x:si>
-    <x:t>0</x:t>
-  </x:si>
-  <x:si>
-    <x:t>225100024</x:t>
-  </x:si>
-  <x:si>
-    <x:t>XT901WZ1140</x:t>
+    <x:t>RC31254</x:t>
+  </x:si>
+  <x:si>
+    <x:t>225100011</x:t>
+  </x:si>
+  <x:si>
+    <x:t>wxt1000jx203</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31255</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31256</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31257</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31258</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31259</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31260</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31261</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31262</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31263</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31264</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31265</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31266</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31267</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31268</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31269</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31270</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31271</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31272</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31273</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31274</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31275</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31276</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31277</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31278</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31279</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31280</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31281</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31282</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31283</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31284</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31285</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31286</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31287</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31288</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31289</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31290</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31291</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31292</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31293</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31294</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31295</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31296</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31297</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31298</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31299</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31300</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31301</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31302</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC31303</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -457,10 +604,10 @@
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.853482" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="6.567768" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.567768" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="5.853482" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="10.282054" style="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12.996339" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="6.424911" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="9.567768" style="0" customWidth="1"/>
     <x:col min="13" max="13" width="18.853482" style="0" customWidth="1"/>
@@ -544,10 +691,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>0</x:v>
@@ -579,16 +726,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>0</x:v>
@@ -620,16 +767,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H4" s="0">
         <x:v>0</x:v>
@@ -661,16 +808,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E5" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H5" s="0">
         <x:v>0</x:v>
@@ -702,16 +849,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H6" s="0">
         <x:v>0</x:v>
@@ -743,16 +890,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E7" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H7" s="0">
         <x:v>0</x:v>
@@ -784,16 +931,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E8" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H8" s="0">
         <x:v>0</x:v>
@@ -825,16 +972,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E9" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H9" s="0">
         <x:v>0</x:v>
@@ -866,16 +1013,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E10" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H10" s="0">
         <x:v>0</x:v>
@@ -907,16 +1054,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H11" s="0">
         <x:v>0</x:v>
@@ -948,16 +1095,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E12" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H12" s="0">
         <x:v>0</x:v>
@@ -989,16 +1136,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E13" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H13" s="0">
         <x:v>0</x:v>
@@ -1030,16 +1177,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E14" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H14" s="0">
         <x:v>0</x:v>
@@ -1071,16 +1218,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E15" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H15" s="0">
         <x:v>0</x:v>
@@ -1112,16 +1259,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H16" s="0">
         <x:v>0</x:v>
@@ -1153,16 +1300,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E17" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H17" s="0">
         <x:v>0</x:v>
@@ -1194,16 +1341,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E18" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H18" s="0">
         <x:v>0</x:v>
@@ -1235,16 +1382,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E19" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H19" s="0">
         <x:v>0</x:v>
@@ -1276,16 +1423,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E20" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H20" s="0">
         <x:v>0</x:v>
@@ -1317,16 +1464,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H21" s="0">
         <x:v>0</x:v>
@@ -1358,16 +1505,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E22" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H22" s="0">
         <x:v>0</x:v>
@@ -1399,16 +1546,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E23" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H23" s="0">
         <x:v>0</x:v>
@@ -1440,16 +1587,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E24" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H24" s="0">
         <x:v>0</x:v>
@@ -1481,16 +1628,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E25" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H25" s="0">
         <x:v>0</x:v>
@@ -1522,16 +1669,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H26" s="0">
         <x:v>0</x:v>
@@ -1563,16 +1710,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E27" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H27" s="0">
         <x:v>0</x:v>
@@ -1604,16 +1751,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E28" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H28" s="0">
         <x:v>0</x:v>
@@ -1645,16 +1792,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E29" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H29" s="0">
         <x:v>0</x:v>
@@ -1686,16 +1833,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E30" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H30" s="0">
         <x:v>0</x:v>
@@ -1727,16 +1874,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H31" s="0">
         <x:v>0</x:v>
@@ -1768,16 +1915,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E32" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F32" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G32" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H32" s="0">
         <x:v>0</x:v>
@@ -1809,16 +1956,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E33" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F33" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G33" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H33" s="0">
         <x:v>0</x:v>
@@ -1850,16 +1997,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="E34" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F34" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G34" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H34" s="0">
         <x:v>0</x:v>
@@ -1891,16 +2038,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E35" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F35" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G35" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H35" s="0">
         <x:v>0</x:v>
@@ -1932,16 +2079,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E36" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F36" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G36" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H36" s="0">
         <x:v>0</x:v>
@@ -1973,16 +2120,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E37" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F37" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G37" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H37" s="0">
         <x:v>0</x:v>
@@ -2014,16 +2161,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E38" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F38" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G38" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H38" s="0">
         <x:v>0</x:v>
@@ -2055,16 +2202,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E39" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F39" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G39" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H39" s="0">
         <x:v>0</x:v>
@@ -2096,16 +2243,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E40" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F40" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G40" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H40" s="0">
         <x:v>0</x:v>
@@ -2137,16 +2284,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E41" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F41" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G41" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H41" s="0">
         <x:v>0</x:v>
@@ -2178,16 +2325,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E42" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F42" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G42" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H42" s="0">
         <x:v>0</x:v>
@@ -2219,16 +2366,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E43" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F43" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G43" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H43" s="0">
         <x:v>0</x:v>
@@ -2260,16 +2407,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E44" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F44" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G44" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H44" s="0">
         <x:v>0</x:v>
@@ -2301,16 +2448,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E45" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F45" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G45" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H45" s="0">
         <x:v>0</x:v>
@@ -2342,16 +2489,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E46" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F46" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G46" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H46" s="0">
         <x:v>0</x:v>
@@ -2383,16 +2530,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="E47" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F47" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G47" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H47" s="0">
         <x:v>0</x:v>
@@ -2424,16 +2571,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E48" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F48" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G48" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H48" s="0">
         <x:v>0</x:v>
@@ -2465,16 +2612,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E49" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F49" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G49" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H49" s="0">
         <x:v>0</x:v>
@@ -2506,16 +2653,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D50" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E50" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F50" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G50" s="0">
-        <x:v>252</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H50" s="0">
         <x:v>0</x:v>
@@ -2547,16 +2694,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D51" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E51" s="0">
-        <x:v>19.4</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="F51" s="0">
-        <x:v>2100</x:v>
+        <x:v>1900</x:v>
       </x:c>
       <x:c r="G51" s="0">
-        <x:v>488.88</x:v>
+        <x:v>444.6</x:v>
       </x:c>
       <x:c r="H51" s="0">
         <x:v>0</x:v>

</xml_diff>

<commit_message>
trabajos con la orden de cortes agregar funcionalidad de configuracion de las vueltas
</commit_message>
<xml_diff>
--- a/bin/Debug/net9.0-windows/RollosCortados.xlsx
+++ b/bin/Debug/net9.0-windows/RollosCortados.xlsx
@@ -73,124 +73,142 @@
     <x:t>tipo_mov</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">02176                                             </x:t>
-  </x:si>
-  <x:si>
-    <x:t>RI-757/40 PP CAVITATED TC8 AP901 WG62</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33552</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14809001</x:t>
-  </x:si>
-  <x:si>
-    <x:t>XX80</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33553</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33554</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33555</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33556</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33557</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33558</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33559</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33560</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33561</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33562</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33563</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33564</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33565</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33566</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33567</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33568</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33569</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33570</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33571</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33572</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33573</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33574</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33575</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33576</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33577</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33578</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33579</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33580</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33581</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33582</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33583</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33584</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33585</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33586</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RC33587</x:t>
+    <x:t xml:space="preserve">02102                    </x:t>
+  </x:si>
+  <x:si>
+    <x:t>RI-757/60 PP CAVITATED TC8 AP901 WG62</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35237</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11584000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>n/a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35238</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35239</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35240</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35241</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35242</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35243</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35244</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35245</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35246</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35247</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35248</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35249</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35250</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35251</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35252</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35253</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35254</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35255</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35256</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35257</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35258</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35259</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35260</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35261</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35262</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35263</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35264</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35265</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35266</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35267</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35268</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35269</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35270</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35271</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35272</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35273</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35274</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35275</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RC35276</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -556,16 +574,16 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:S37"/>
+  <x:dimension ref="A1:S41"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="26.424911" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="38.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.853482" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="5.567768" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="4.139196" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="5.853482" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="9.282054" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="12.996339" style="0" customWidth="1"/>
@@ -656,10 +674,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>0</x:v>
@@ -667,17 +685,23 @@
       <x:c r="I2" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J2" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M2" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N2" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O2" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P2" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q2" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R2" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:19">
@@ -691,16 +715,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>0</x:v>
@@ -708,17 +732,23 @@
       <x:c r="I3" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J3" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M3" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N3" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O3" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P3" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q3" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R3" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:19">
@@ -732,16 +762,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H4" s="0">
         <x:v>0</x:v>
@@ -749,17 +779,23 @@
       <x:c r="I4" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J4" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M4" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N4" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O4" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P4" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q4" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R4" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:19">
@@ -773,16 +809,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E5" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H5" s="0">
         <x:v>0</x:v>
@@ -790,17 +826,23 @@
       <x:c r="I5" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J5" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M5" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N5" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O5" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P5" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q5" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R5" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:19">
@@ -814,16 +856,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E6" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H6" s="0">
         <x:v>0</x:v>
@@ -831,17 +873,23 @@
       <x:c r="I6" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J6" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M6" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N6" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P6" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q6" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R6" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:19">
@@ -855,16 +903,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E7" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H7" s="0">
         <x:v>0</x:v>
@@ -872,17 +920,23 @@
       <x:c r="I7" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J7" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M7" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N7" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O7" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P7" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q7" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R7" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:19">
@@ -896,16 +950,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E8" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H8" s="0">
         <x:v>0</x:v>
@@ -913,17 +967,23 @@
       <x:c r="I8" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J8" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M8" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N8" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O8" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P8" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q8" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R8" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:19">
@@ -937,16 +997,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E9" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H9" s="0">
         <x:v>0</x:v>
@@ -954,17 +1014,23 @@
       <x:c r="I9" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J9" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M9" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N9" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O9" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P9" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q9" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R9" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:19">
@@ -978,16 +1044,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E10" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H10" s="0">
         <x:v>0</x:v>
@@ -995,17 +1061,23 @@
       <x:c r="I10" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J10" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M10" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N10" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O10" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P10" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q10" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R10" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:19">
@@ -1019,16 +1091,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E11" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H11" s="0">
         <x:v>0</x:v>
@@ -1036,17 +1108,23 @@
       <x:c r="I11" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J11" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M11" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N11" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O11" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P11" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q11" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R11" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:19">
@@ -1060,16 +1138,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E12" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H12" s="0">
         <x:v>0</x:v>
@@ -1077,17 +1155,23 @@
       <x:c r="I12" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J12" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M12" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N12" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O12" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P12" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q12" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R12" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:19">
@@ -1101,16 +1185,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E13" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H13" s="0">
         <x:v>0</x:v>
@@ -1118,17 +1202,23 @@
       <x:c r="I13" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J13" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M13" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N13" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O13" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P13" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q13" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R13" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:19">
@@ -1142,16 +1232,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E14" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H14" s="0">
         <x:v>0</x:v>
@@ -1159,17 +1249,23 @@
       <x:c r="I14" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J14" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M14" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N14" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O14" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P14" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q14" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R14" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:19">
@@ -1183,16 +1279,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E15" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H15" s="0">
         <x:v>0</x:v>
@@ -1200,17 +1296,23 @@
       <x:c r="I15" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J15" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M15" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N15" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O15" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P15" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q15" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R15" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:19">
@@ -1224,16 +1326,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E16" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H16" s="0">
         <x:v>0</x:v>
@@ -1241,17 +1343,23 @@
       <x:c r="I16" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J16" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M16" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N16" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O16" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P16" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q16" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R16" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:19">
@@ -1265,16 +1373,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E17" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H17" s="0">
         <x:v>0</x:v>
@@ -1282,17 +1390,23 @@
       <x:c r="I17" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J17" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M17" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N17" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O17" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P17" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q17" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R17" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:19">
@@ -1306,16 +1420,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E18" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H18" s="0">
         <x:v>0</x:v>
@@ -1323,17 +1437,23 @@
       <x:c r="I18" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J18" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M18" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N18" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O18" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P18" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q18" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R18" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:19">
@@ -1347,16 +1467,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E19" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H19" s="0">
         <x:v>0</x:v>
@@ -1364,17 +1484,23 @@
       <x:c r="I19" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J19" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M19" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N19" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O19" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P19" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q19" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R19" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:19">
@@ -1388,16 +1514,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E20" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H20" s="0">
         <x:v>0</x:v>
@@ -1405,17 +1531,23 @@
       <x:c r="I20" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J20" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M20" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N20" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O20" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P20" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q20" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R20" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:19">
@@ -1429,16 +1561,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E21" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H21" s="0">
         <x:v>0</x:v>
@@ -1446,17 +1578,23 @@
       <x:c r="I21" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J21" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M21" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N21" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O21" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P21" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q21" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R21" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:19">
@@ -1470,16 +1608,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E22" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H22" s="0">
         <x:v>0</x:v>
@@ -1487,17 +1625,23 @@
       <x:c r="I22" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J22" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M22" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N22" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O22" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P22" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q22" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R22" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:19">
@@ -1511,16 +1655,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E23" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H23" s="0">
         <x:v>0</x:v>
@@ -1528,17 +1672,23 @@
       <x:c r="I23" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J23" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M23" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N23" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O23" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P23" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q23" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R23" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:19">
@@ -1552,16 +1702,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E24" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H24" s="0">
         <x:v>0</x:v>
@@ -1569,17 +1719,23 @@
       <x:c r="I24" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J24" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M24" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N24" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O24" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P24" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q24" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R24" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:19">
@@ -1593,16 +1749,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E25" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H25" s="0">
         <x:v>0</x:v>
@@ -1610,17 +1766,23 @@
       <x:c r="I25" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J25" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M25" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N25" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O25" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P25" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q25" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R25" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:19">
@@ -1634,16 +1796,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E26" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H26" s="0">
         <x:v>0</x:v>
@@ -1651,17 +1813,23 @@
       <x:c r="I26" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J26" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M26" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N26" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O26" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P26" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q26" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R26" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:19">
@@ -1675,16 +1843,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E27" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H27" s="0">
         <x:v>0</x:v>
@@ -1692,17 +1860,23 @@
       <x:c r="I27" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J27" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M27" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N27" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O27" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P27" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q27" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R27" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:19">
@@ -1716,16 +1890,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E28" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H28" s="0">
         <x:v>0</x:v>
@@ -1733,17 +1907,23 @@
       <x:c r="I28" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J28" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M28" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N28" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O28" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P28" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q28" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R28" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:19">
@@ -1757,16 +1937,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E29" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H29" s="0">
         <x:v>0</x:v>
@@ -1774,17 +1954,23 @@
       <x:c r="I29" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J29" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M29" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N29" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O29" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P29" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q29" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R29" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:19">
@@ -1798,16 +1984,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E30" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H30" s="0">
         <x:v>0</x:v>
@@ -1815,17 +2001,23 @@
       <x:c r="I30" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J30" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M30" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N30" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O30" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P30" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q30" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R30" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:19">
@@ -1839,16 +2031,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="E31" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H31" s="0">
         <x:v>0</x:v>
@@ -1856,17 +2048,23 @@
       <x:c r="I31" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J31" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M31" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N31" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O31" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P31" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q31" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R31" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:19">
@@ -1880,16 +2078,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E32" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F32" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G32" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H32" s="0">
         <x:v>0</x:v>
@@ -1897,17 +2095,23 @@
       <x:c r="I32" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J32" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M32" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N32" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O32" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P32" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q32" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R32" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:19">
@@ -1921,16 +2125,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E33" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F33" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G33" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H33" s="0">
         <x:v>0</x:v>
@@ -1938,17 +2142,23 @@
       <x:c r="I33" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J33" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M33" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O33" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P33" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q33" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R33" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:19">
@@ -1962,16 +2172,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E34" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F34" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G34" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H34" s="0">
         <x:v>0</x:v>
@@ -1979,17 +2189,23 @@
       <x:c r="I34" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J34" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M34" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N34" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O34" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P34" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q34" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R34" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:19">
@@ -2003,16 +2219,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E35" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F35" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G35" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H35" s="0">
         <x:v>0</x:v>
@@ -2020,17 +2236,23 @@
       <x:c r="I35" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J35" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M35" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N35" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O35" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P35" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q35" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R35" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:19">
@@ -2044,16 +2266,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E36" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F36" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G36" s="0">
-        <x:v>252</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H36" s="0">
         <x:v>0</x:v>
@@ -2061,17 +2283,23 @@
       <x:c r="I36" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J36" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M36" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N36" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O36" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P36" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q36" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R36" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:19">
@@ -2085,16 +2313,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E37" s="0">
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="F37" s="0">
-        <x:v>2100</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G37" s="0">
-        <x:v>239.4</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="H37" s="0">
         <x:v>0</x:v>
@@ -2102,17 +2330,211 @@
       <x:c r="I37" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="J37" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
       <x:c r="M37" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N37" s="0">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="O37" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P37" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="Q37" s="0" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="R37" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" spans="1:19">
+      <x:c r="A38" s="0">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B38" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C38" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D38" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="E38" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F38" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G38" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I38" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O38" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P38" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q38" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R38" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" spans="1:19">
+      <x:c r="A39" s="0">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B39" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C39" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D39" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E39" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F39" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G39" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I39" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O39" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P39" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q39" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R39" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" spans="1:19">
+      <x:c r="A40" s="0">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B40" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C40" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D40" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E40" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F40" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G40" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I40" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O40" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P40" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q40" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R40" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" spans="1:19">
+      <x:c r="A41" s="0">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B41" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C41" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D41" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E41" s="0">
+        <x:v>9.5</x:v>
+      </x:c>
+      <x:c r="F41" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G41" s="0">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="H41" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I41" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M41" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N41" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O41" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="P41" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="Q41" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R41" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
trabajos con la carga de los datos en la oc, mejora en las tareas asincronas al cargar
</commit_message>
<xml_diff>
--- a/bin/Debug/net9.0-windows/RollosCortados.xlsx
+++ b/bin/Debug/net9.0-windows/RollosCortados.xlsx
@@ -76,16 +76,16 @@
     <x:t>vuelta</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">6770                                              </x:t>
+    <x:t xml:space="preserve">7836                                              </x:t>
   </x:si>
   <x:si>
-    <x:t>Coated 80 AP904 SK60</x:t>
+    <x:t>07836 (Thermal top AP-903 WG56....)</x:t>
   </x:si>
   <x:si>
     <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t>224091024</x:t>
+    <x:t>225009002</x:t>
   </x:si>
   <x:si>
     <x:t>N/A</x:t>
@@ -454,16 +454,16 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:T6"/>
+  <x:dimension ref="A1:T51"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="25.853482" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="33.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.853482" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="4.996339" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.567768" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="5.853482" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="10.282054" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="12.996339" style="0" customWidth="1"/>
@@ -558,10 +558,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>5000</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>600</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>0</x:v>
@@ -602,10 +602,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>5000</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>600</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>0</x:v>
@@ -646,10 +646,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>5000</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>600</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H4" s="0">
         <x:v>0</x:v>
@@ -690,10 +690,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>5000</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>600</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="H5" s="0">
         <x:v>0</x:v>
@@ -734,10 +734,10 @@
         <x:v>19.4</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>5000</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>1164</x:v>
+        <x:v>465.6</x:v>
       </x:c>
       <x:c r="H6" s="0">
         <x:v>0</x:v>
@@ -758,6 +758,1986 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="T6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:20">
+      <x:c r="A7" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E7" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F7" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G7" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H7" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J7" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M7" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N7" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q7" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T7" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:20">
+      <x:c r="A8" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E8" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F8" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G8" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J8" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q8" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:20">
+      <x:c r="A9" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E9" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F9" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G9" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H9" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J9" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M9" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N9" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q9" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T9" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:20">
+      <x:c r="A10" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E10" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F10" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G10" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H10" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J10" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M10" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q10" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T10" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:20">
+      <x:c r="A11" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E11" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F11" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G11" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H11" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J11" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M11" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q11" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T11" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:20">
+      <x:c r="A12" s="0">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E12" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F12" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G12" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H12" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J12" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M12" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q12" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T12" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:20">
+      <x:c r="A13" s="0">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E13" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F13" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G13" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H13" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J13" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M13" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q13" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T13" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:20">
+      <x:c r="A14" s="0">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E14" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F14" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G14" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H14" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J14" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M14" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N14" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q14" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T14" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:20">
+      <x:c r="A15" s="0">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C15" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D15" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E15" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F15" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G15" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H15" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J15" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M15" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N15" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q15" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T15" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:20">
+      <x:c r="A16" s="0">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B16" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C16" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D16" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E16" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F16" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G16" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H16" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J16" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M16" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N16" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q16" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T16" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:20">
+      <x:c r="A17" s="0">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C17" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D17" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E17" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F17" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G17" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H17" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J17" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M17" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N17" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q17" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T17" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:20">
+      <x:c r="A18" s="0">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C18" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D18" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E18" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F18" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G18" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H18" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J18" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M18" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N18" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q18" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T18" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:20">
+      <x:c r="A19" s="0">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C19" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D19" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E19" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F19" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G19" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H19" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J19" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M19" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N19" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q19" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T19" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:20">
+      <x:c r="A20" s="0">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C20" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D20" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E20" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F20" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G20" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H20" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J20" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M20" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N20" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q20" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T20" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:20">
+      <x:c r="A21" s="0">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B21" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C21" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D21" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E21" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F21" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G21" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H21" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J21" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M21" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N21" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q21" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T21" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:20">
+      <x:c r="A22" s="0">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B22" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C22" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D22" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E22" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F22" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G22" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H22" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J22" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M22" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N22" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q22" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T22" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:20">
+      <x:c r="A23" s="0">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B23" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C23" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D23" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E23" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F23" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G23" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H23" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J23" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M23" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N23" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q23" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T23" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:20">
+      <x:c r="A24" s="0">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B24" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C24" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D24" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E24" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F24" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G24" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H24" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J24" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M24" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N24" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q24" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T24" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:20">
+      <x:c r="A25" s="0">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C25" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D25" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E25" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F25" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G25" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H25" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I25" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J25" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M25" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N25" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q25" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T25" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:20">
+      <x:c r="A26" s="0">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C26" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D26" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E26" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F26" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G26" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H26" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I26" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J26" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M26" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N26" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q26" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T26" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:20">
+      <x:c r="A27" s="0">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B27" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C27" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D27" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E27" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F27" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G27" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H27" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I27" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J27" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M27" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N27" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q27" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T27" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:20">
+      <x:c r="A28" s="0">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B28" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C28" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D28" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E28" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F28" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G28" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H28" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J28" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M28" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N28" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q28" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T28" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:20">
+      <x:c r="A29" s="0">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B29" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C29" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D29" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E29" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F29" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G29" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H29" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J29" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M29" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N29" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q29" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T29" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:20">
+      <x:c r="A30" s="0">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B30" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C30" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D30" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E30" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F30" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G30" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H30" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J30" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M30" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N30" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q30" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T30" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:20">
+      <x:c r="A31" s="0">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B31" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C31" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D31" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E31" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F31" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G31" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H31" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J31" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M31" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N31" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q31" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T31" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" spans="1:20">
+      <x:c r="A32" s="0">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B32" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C32" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D32" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E32" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F32" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G32" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H32" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J32" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M32" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N32" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q32" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T32" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" spans="1:20">
+      <x:c r="A33" s="0">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B33" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C33" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D33" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E33" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F33" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G33" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H33" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J33" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M33" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N33" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q33" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T33" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" spans="1:20">
+      <x:c r="A34" s="0">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B34" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C34" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D34" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E34" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F34" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G34" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H34" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J34" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M34" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N34" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q34" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T34" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" spans="1:20">
+      <x:c r="A35" s="0">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B35" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C35" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D35" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E35" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F35" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G35" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H35" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J35" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M35" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N35" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q35" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T35" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" spans="1:20">
+      <x:c r="A36" s="0">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B36" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C36" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D36" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E36" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F36" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G36" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H36" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J36" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M36" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N36" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q36" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T36" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" spans="1:20">
+      <x:c r="A37" s="0">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B37" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C37" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D37" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E37" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F37" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G37" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H37" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I37" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J37" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M37" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N37" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q37" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T37" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" spans="1:20">
+      <x:c r="A38" s="0">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B38" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C38" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D38" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E38" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F38" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G38" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I38" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J38" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q38" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" spans="1:20">
+      <x:c r="A39" s="0">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B39" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C39" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D39" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E39" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F39" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G39" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I39" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J39" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q39" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" spans="1:20">
+      <x:c r="A40" s="0">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B40" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C40" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D40" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E40" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F40" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G40" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I40" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J40" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q40" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" spans="1:20">
+      <x:c r="A41" s="0">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B41" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C41" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D41" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E41" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F41" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G41" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H41" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I41" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J41" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M41" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N41" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q41" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T41" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" spans="1:20">
+      <x:c r="A42" s="0">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B42" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C42" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D42" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E42" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F42" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G42" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H42" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I42" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J42" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M42" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q42" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T42" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" spans="1:20">
+      <x:c r="A43" s="0">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B43" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C43" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D43" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E43" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F43" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G43" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H43" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I43" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J43" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M43" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N43" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q43" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T43" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" spans="1:20">
+      <x:c r="A44" s="0">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B44" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C44" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D44" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E44" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F44" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G44" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H44" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I44" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J44" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M44" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N44" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q44" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T44" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" spans="1:20">
+      <x:c r="A45" s="0">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B45" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C45" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D45" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E45" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F45" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G45" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H45" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I45" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J45" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M45" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N45" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q45" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T45" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" spans="1:20">
+      <x:c r="A46" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B46" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C46" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D46" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E46" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F46" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G46" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H46" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I46" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J46" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M46" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N46" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q46" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T46" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" spans="1:20">
+      <x:c r="A47" s="0">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B47" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C47" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D47" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E47" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F47" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G47" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H47" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I47" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J47" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M47" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N47" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q47" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T47" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" spans="1:20">
+      <x:c r="A48" s="0">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B48" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C48" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D48" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E48" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F48" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G48" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H48" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I48" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J48" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M48" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N48" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q48" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T48" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" spans="1:20">
+      <x:c r="A49" s="0">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B49" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C49" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D49" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E49" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F49" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G49" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H49" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I49" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J49" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M49" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N49" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q49" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T49" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" spans="1:20">
+      <x:c r="A50" s="0">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B50" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C50" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D50" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E50" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F50" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G50" s="0">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H50" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I50" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J50" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M50" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N50" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q50" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T50" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" spans="1:20">
+      <x:c r="A51" s="0">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B51" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C51" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D51" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E51" s="0">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="F51" s="0">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G51" s="0">
+        <x:v>465.6</x:v>
+      </x:c>
+      <x:c r="H51" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I51" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J51" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="M51" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N51" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q51" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T51" s="0">
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>